<commit_message>
Release round-5 statistical and reproducibility update
</commit_message>
<xml_diff>
--- a/results/tables/tHRR-I_public_data_results.xlsx
+++ b/results/tables/tHRR-I_public_data_results.xlsx
@@ -2,34 +2,39 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rde40f86ed25a43a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction performance" sheetId="2" r:id="R3c612935666c4964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction comparisons" sheetId="3" r:id="Rfa20b8268a2e4269"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Within-person summary" sheetId="4" r:id="Rd43c2d9230364a69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant associations" sheetId="5" r:id="Ree9b0008790348f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discretization" sheetId="6" r:id="R30725bc87e174aa5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeated splits summary" sheetId="7" r:id="R83932f81b2ac4fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeated splits" sheetId="8" r:id="R197199db3bb14607"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching stability" sheetId="9" r:id="R7164591f809441e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High RPE balanced" sheetId="10" r:id="R76245abdc79e4006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High RPE participant" sheetId="11" r:id="Rf7dcd64dedeb4e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ordinal sensitivity" sheetId="12" r:id="R9e576224f9cf491c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HRR clipping" sheetId="13" r:id="R2d862d0bb17c40d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction range" sheetId="14" r:id="R31b3e2b568994afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equal-mean examples" sheetId="15" r:id="R7d379f069b0b462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw signal anchors" sheetId="16" r:id="R0447b8908c6e4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching model performance" sheetId="17" r:id="R24b5e2b4937c43c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weight profile" sheetId="18" r:id="R9f612ae7e99144c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant anchors" sheetId="19" r:id="R957c16fa2eca4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selection aware" sheetId="20" r:id="R6847d934b20d4aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching confidence" sheetId="21" r:id="R5d8f46733fde4d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lambda heterogeneity" sheetId="22" r:id="Rcb48ec60a0b04dd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE repeated measures" sheetId="23" r:id="Rf640f6b88e0f4fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE agreement" sheetId="24" r:id="Rbf2d5df6188d4264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE agreement intervals" sheetId="25" r:id="Rc2e075705c184385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE synchronization" sheetId="26" r:id="Rf2a81f0554064dc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Malaga endpoint sensitivity" sheetId="27" r:id="R52a2202dcfee426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Malaga anchor sensitivity" sheetId="28" r:id="Re1b0523768b74030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R0370997591664146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction performance" sheetId="2" r:id="Rc271e24dd2e141af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction comparisons" sheetId="3" r:id="R7d76022ae85c42b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Within-person summary" sheetId="4" r:id="R2fbea52212a6451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant associations" sheetId="5" r:id="R7e1532104b98410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discretization" sheetId="6" r:id="Rf65fc2fba687410e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeated splits summary" sheetId="7" r:id="R230b9996939e4644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Repeated splits" sheetId="8" r:id="R81fde0cd68e0444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching stability" sheetId="9" r:id="Rd9152d637f4e4aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High RPE balanced" sheetId="10" r:id="R6360094dd31145cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High RPE participant" sheetId="11" r:id="R8179f10258994c3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ordinal sensitivity" sheetId="12" r:id="Rfcb154cc1e1b41c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HRR clipping" sheetId="13" r:id="R443d2dda25534a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prediction range" sheetId="14" r:id="Rc767f6481a9f4752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equal-mean examples" sheetId="15" r:id="R09b3cf5fdbb74af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw signal anchors" sheetId="16" r:id="Rd745448066304e2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching model performance" sheetId="17" r:id="R197f680c70514c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weight profile" sheetId="18" r:id="Rbe2ae7ffac654985"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant anchors" sheetId="19" r:id="R740135567b53422d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Selection aware" sheetId="20" r:id="Ra21be65c5e594c24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matching confidence" sheetId="21" r:id="Rc5306615c86948b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lambda heterogeneity" sheetId="22" r:id="R8ce05eaca8464e4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE repeated measures" sheetId="23" r:id="R30a1d8554b2944b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE agreement" sheetId="24" r:id="R9ee5eda159a946e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE agreement intervals" sheetId="25" r:id="R3c04724d05714778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE synchronization" sheetId="26" r:id="R79630916f86f4640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Malaga endpoint sensitivity" sheetId="27" r:id="R4a5b98e5a3e940e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Malaga anchor sensitivity" sheetId="28" r:id="Rd0f710fe6153406b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round5_Incremental" sheetId="29" r:id="R362e557402824000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round5_ParticipantLoss" sheetId="30" r:id="R1cdb510d42084322"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round5_SampleFlow" sheetId="31" r:id="R23ce3313cab549c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE_RM_Agreement" sheetId="32" r:id="R90ed404f4c9446a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WEEE_StageFlow" sheetId="33" r:id="R93c425a859e54f4a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40,11 +45,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="164" formatCode="0.0000"/>
     <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="0.000"/>
+    <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -75,8 +82,43 @@
       <x:color rgb="FF007C91"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="8"/>
+      <x:color rgb="FF1F2937"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -113,8 +155,28 @@
         <x:fgColor rgb="FFEAF3F6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F6B78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDEFEF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="4">
+  <x:borders count="5">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -146,11 +208,25 @@
         <x:color rgb="FF1E3F66"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB7C9D6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB7C9D6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB7C9D6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9D6"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -311,6 +387,35 @@
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -635,7 +740,7 @@
         <x:v>Development status</x:v>
       </x:c>
       <x:c r="B4" s="64" t="str">
-        <x:v>Exploratory PMData method development; principal comparison was not preregistered</x:v>
+        <x:v>Exploratory PMData formula development; the round-5 outer-fold comparison was not preregistered</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -643,7 +748,7 @@
         <x:v>Selection-aware result</x:v>
       </x:c>
       <x:c r="B5" s="41" t="str">
-        <x:v>Outer LOPO reselected family and parameter: ΔMAE -0.094 RPE units (95% CI -0.161 to -0.031)</x:v>
+        <x:v>Mean HRR + Δtilt versus mean HRR: ΔMAE -0.070 RPE units (-0.165 to 0.035); exact P=0.228</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -683,7 +788,7 @@
         <x:v>Zephyr agreement</x:v>
       </x:c>
       <x:c r="B10" s="64" t="str">
-        <x:v>tHRR-I ICC(A,1) 0.854 (0.667 to 0.952); limits of agreement -0.257 to 0.205</x:v>
+        <x:v>Zephyr tHRR-I participant-balanced CCC 0.846 (0.654 to 0.946); repeated-measures limits -0.262 to 0.213</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -699,7 +804,7 @@
         <x:v>Practical interpretation</x:v>
       </x:c>
       <x:c r="B12" s="64" t="str">
-        <x:v>Candidate retrospective session-review descriptor; not a prescription, alert, or clinical measure</x:v>
+        <x:v>Research-level retrospective session descriptor; not a prescription, alert, or clinical measure</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -707,7 +812,7 @@
         <x:v>Uncertainty</x:v>
       </x:c>
       <x:c r="B13" s="41" t="str">
-        <x:v>Participant-cluster intervals; formula-invention optimism remains in PMData</x:v>
+        <x:v>Participant-cluster intervals; model-family invention and fixed-λ sensitivities remain development-sample conditional</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -723,7 +828,7 @@
         <x:v>Software</x:v>
       </x:c>
       <x:c r="B15" s="41" t="str">
-        <x:v>Python 3.12.13; pandas 2.2.3; NumPy 2.3.5; openpyxl 3.1.5</x:v>
+        <x:v>Analysis: Python 3.12.13, pandas 2.2.3, NumPy 2.3.5; workbook assembly: @oai/artifact-tool 2.8.6+</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8204,6 +8309,450 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="29" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="B1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="C1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="D1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="E1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="F1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="G1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="H1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="I1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="J1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="K1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+      <x:c r="L1" s="67" t="str">
+        <x:v>Round 5: participant-grouped model comparison</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="F2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="G2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="H2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="I2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="J2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="K2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+      <x:c r="L2" s="70" t="str">
+        <x:v>Negative ΔMAE favors the candidate. Participant is the independent resampling unit. Fixed-λ rows are development-condition sensitivities.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>Model</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>Participants</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>Participant-balanced MAE</x:v>
+      </x:c>
+      <x:c r="D4" s="75" t="str">
+        <x:v>ΔMAE vs mean HRR</x:v>
+      </x:c>
+      <x:c r="E4" s="75" t="str">
+        <x:v>Relative MAE change (%)</x:v>
+      </x:c>
+      <x:c r="F4" s="75" t="str">
+        <x:v>Bootstrap lower</x:v>
+      </x:c>
+      <x:c r="G4" s="75" t="str">
+        <x:v>Bootstrap upper</x:v>
+      </x:c>
+      <x:c r="H4" s="75" t="str">
+        <x:v>Exact sign-flip P</x:v>
+      </x:c>
+      <x:c r="I4" s="75" t="str">
+        <x:v>Favor candidate (n)</x:v>
+      </x:c>
+      <x:c r="J4" s="75" t="str">
+        <x:v>Favor base (n)</x:v>
+      </x:c>
+      <x:c r="K4" s="75" t="str">
+        <x:v>Leave-one-out Δ min</x:v>
+      </x:c>
+      <x:c r="L4" s="75" t="str">
+        <x:v>Leave-one-out Δ max</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="76" t="str">
+        <x:v>Mean HRR</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C5" s="77" t="n">
+        <x:v>1.3020464195357122</x:v>
+      </x:c>
+      <x:c r="D5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="78" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="77"/>
+      <x:c r="I5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L5" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="76" t="str">
+        <x:v>Mean HRR + variance</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C6" s="77" t="n">
+        <x:v>1.2937751659446943</x:v>
+      </x:c>
+      <x:c r="D6" s="77" t="n">
+        <x:v>-0.008271253591017621</x:v>
+      </x:c>
+      <x:c r="E6" s="78" t="n">
+        <x:v>-0.6352502850065062</x:v>
+      </x:c>
+      <x:c r="F6" s="77" t="n">
+        <x:v>-0.0640127908795715</x:v>
+      </x:c>
+      <x:c r="G6" s="77" t="n">
+        <x:v>0.05372513314046594</x:v>
+      </x:c>
+      <x:c r="H6" s="77" t="n">
+        <x:v>0.798095703125</x:v>
+      </x:c>
+      <x:c r="I6" s="77" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J6" s="77" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K6" s="77" t="n">
+        <x:v>-0.02867709835210867</x:v>
+      </x:c>
+      <x:c r="L6" s="77" t="n">
+        <x:v>0.00488033152080007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="76" t="str">
+        <x:v>Mean HRR + time ≥80% HRR</x:v>
+      </x:c>
+      <x:c r="B7" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C7" s="77" t="n">
+        <x:v>1.2789399577902902</x:v>
+      </x:c>
+      <x:c r="D7" s="77" t="n">
+        <x:v>-0.023106461745421726</x:v>
+      </x:c>
+      <x:c r="E7" s="78" t="n">
+        <x:v>-1.7746265723507078</x:v>
+      </x:c>
+      <x:c r="F7" s="77" t="n">
+        <x:v>-0.13557657143293464</x:v>
+      </x:c>
+      <x:c r="G7" s="77" t="n">
+        <x:v>0.10695448726255276</x:v>
+      </x:c>
+      <x:c r="H7" s="77" t="n">
+        <x:v>0.7205810546875</x:v>
+      </x:c>
+      <x:c r="I7" s="77" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J7" s="77" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K7" s="77" t="n">
+        <x:v>-0.05758196383070456</x:v>
+      </x:c>
+      <x:c r="L7" s="77" t="n">
+        <x:v>-0.00044134386031396966</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="76" t="str">
+        <x:v>Mean HRR + Δtilt, fixed λ=6.2</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C8" s="77" t="n">
+        <x:v>1.2282576049993592</x:v>
+      </x:c>
+      <x:c r="D8" s="77" t="n">
+        <x:v>-0.0737888145363529</x:v>
+      </x:c>
+      <x:c r="E8" s="78" t="n">
+        <x:v>-5.667141618703943</x:v>
+      </x:c>
+      <x:c r="F8" s="77" t="n">
+        <x:v>-0.15494498038670443</x:v>
+      </x:c>
+      <x:c r="G8" s="77" t="n">
+        <x:v>0.0017989210274185934</x:v>
+      </x:c>
+      <x:c r="H8" s="77" t="n">
+        <x:v>0.09844970703125</x:v>
+      </x:c>
+      <x:c r="I8" s="77" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="J8" s="77" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K8" s="77" t="n">
+        <x:v>-0.09104035335025747</x:v>
+      </x:c>
+      <x:c r="L8" s="77" t="n">
+        <x:v>-0.04984219599314725</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="76" t="str">
+        <x:v>tHRR-I alone, fixed λ=6.2</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C9" s="77" t="n">
+        <x:v>1.2276748933553887</x:v>
+      </x:c>
+      <x:c r="D9" s="77" t="n">
+        <x:v>-0.07437152618032332</x:v>
+      </x:c>
+      <x:c r="E9" s="78" t="n">
+        <x:v>-5.7118951417141455</x:v>
+      </x:c>
+      <x:c r="F9" s="77" t="n">
+        <x:v>-0.13308062840882492</x:v>
+      </x:c>
+      <x:c r="G9" s="77" t="n">
+        <x:v>-0.0171698191090123</x:v>
+      </x:c>
+      <x:c r="H9" s="77" t="n">
+        <x:v>0.02996826171875</x:v>
+      </x:c>
+      <x:c r="I9" s="77" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J9" s="77" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K9" s="77" t="n">
+        <x:v>-0.08466746313466</x:v>
+      </x:c>
+      <x:c r="L9" s="77" t="n">
+        <x:v>-0.059995828595085725</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="76" t="str">
+        <x:v>Mean HRR + Δtilt, nested λ</x:v>
+      </x:c>
+      <x:c r="B10" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C10" s="77" t="n">
+        <x:v>1.2320967470002568</x:v>
+      </x:c>
+      <x:c r="D10" s="77" t="n">
+        <x:v>-0.0699496725354552</x:v>
+      </x:c>
+      <x:c r="E10" s="78" t="n">
+        <x:v>-5.372287153970906</x:v>
+      </x:c>
+      <x:c r="F10" s="77" t="n">
+        <x:v>-0.16544334872389313</x:v>
+      </x:c>
+      <x:c r="G10" s="77" t="n">
+        <x:v>0.03487836821016581</x:v>
+      </x:c>
+      <x:c r="H10" s="77" t="n">
+        <x:v>0.2275390625</x:v>
+      </x:c>
+      <x:c r="I10" s="77" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J10" s="77" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K10" s="77" t="n">
+        <x:v>-0.10906895743010171</x:v>
+      </x:c>
+      <x:c r="L10" s="77" t="n">
+        <x:v>-0.04511976036274091</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="76" t="str">
+        <x:v>Selection-aware transparent pipeline</x:v>
+      </x:c>
+      <x:c r="B11" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C11" s="77" t="n">
+        <x:v>1.2449495567696305</x:v>
+      </x:c>
+      <x:c r="D11" s="77" t="n">
+        <x:v>-0.057096862766081495</x:v>
+      </x:c>
+      <x:c r="E11" s="78" t="n">
+        <x:v>-4.385163378924791</x:v>
+      </x:c>
+      <x:c r="F11" s="77" t="n">
+        <x:v>-0.15098765691397598</x:v>
+      </x:c>
+      <x:c r="G11" s="77" t="n">
+        <x:v>0.04824985027560582</x:v>
+      </x:c>
+      <x:c r="H11" s="77" t="n">
+        <x:v>0.3115234375</x:v>
+      </x:c>
+      <x:c r="I11" s="77" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J11" s="77" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K11" s="77" t="n">
+        <x:v>-0.09529808982005845</x:v>
+      </x:c>
+      <x:c r="L11" s="77" t="n">
+        <x:v>-0.031348892752697644</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" customHeight="1">
+      <x:c r="A13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="B13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="C13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="D13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="E13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="F13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="G13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="H13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="I13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="J13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="K13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+      <x:c r="L13" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_model_performance.csv | Public data: https://datasets.simula.no/pmdata/</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A13:L13"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -8537,6 +9086,2071 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="B1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="C1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="D1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="E1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="F1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="G1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="H1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="I1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+      <x:c r="J1" s="67" t="str">
+        <x:v>Participant-level held-out losses</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="F2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="G2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="H2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="I2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+      <x:c r="J2" s="70" t="str">
+        <x:v>Formulas calculate paired ΔMAE from the archived participant-level MAE columns; negative values favor the candidate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>Participant</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>Sessions</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>Base mean MAE</x:v>
+      </x:c>
+      <x:c r="D4" s="75" t="str">
+        <x:v>Nested Δtilt MAE</x:v>
+      </x:c>
+      <x:c r="E4" s="75" t="str">
+        <x:v>ΔMAE nested</x:v>
+      </x:c>
+      <x:c r="F4" s="75" t="str">
+        <x:v>Fixed Δtilt MAE</x:v>
+      </x:c>
+      <x:c r="G4" s="75" t="str">
+        <x:v>ΔMAE fixed</x:v>
+      </x:c>
+      <x:c r="H4" s="75" t="str">
+        <x:v>Fixed tHRR-I MAE</x:v>
+      </x:c>
+      <x:c r="I4" s="75" t="str">
+        <x:v>ΔMAE stand-alone</x:v>
+      </x:c>
+      <x:c r="J4" s="75" t="str">
+        <x:v>Selected transparent MAE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="76" t="str">
+        <x:v>p01</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C5" s="77" t="n">
+        <x:v>0.6219671675554482</x:v>
+      </x:c>
+      <x:c r="D5" s="77" t="n">
+        <x:v>0.5575996125165622</x:v>
+      </x:c>
+      <x:c r="E5" s="77" t="n">
+        <x:f>D5-C5</x:f>
+        <x:v>-0.06436755503888603</x:v>
+      </x:c>
+      <x:c r="F5" s="77" t="n">
+        <x:v>0.5698426734342089</x:v>
+      </x:c>
+      <x:c r="G5" s="77" t="n">
+        <x:f>F5-C5</x:f>
+        <x:v>-0.05212449412123932</x:v>
+      </x:c>
+      <x:c r="H5" s="77" t="n">
+        <x:v>0.5612905339169952</x:v>
+      </x:c>
+      <x:c r="I5" s="77" t="n">
+        <x:f>H5-C5</x:f>
+        <x:v>-0.06067663363845299</x:v>
+      </x:c>
+      <x:c r="J5" s="77" t="n">
+        <x:v>0.5575996125165622</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="76" t="str">
+        <x:v>p02</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C6" s="77" t="n">
+        <x:v>0.655198327516322</x:v>
+      </x:c>
+      <x:c r="D6" s="77" t="n">
+        <x:v>0.6447678662943364</x:v>
+      </x:c>
+      <x:c r="E6" s="77" t="n">
+        <x:f>D6-C6</x:f>
+        <x:v>-0.010430461221985654</x:v>
+      </x:c>
+      <x:c r="F6" s="77" t="n">
+        <x:v>0.680294520303867</x:v>
+      </x:c>
+      <x:c r="G6" s="77" t="n">
+        <x:f>F6-C6</x:f>
+        <x:v>0.025096192787544935</x:v>
+      </x:c>
+      <x:c r="H6" s="77" t="n">
+        <x:v>0.6741975664405727</x:v>
+      </x:c>
+      <x:c r="I6" s="77" t="n">
+        <x:f>H6-C6</x:f>
+        <x:v>0.018999238924250705</x:v>
+      </x:c>
+      <x:c r="J6" s="77" t="n">
+        <x:v>0.6447678662943364</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="76" t="str">
+        <x:v>p03</x:v>
+      </x:c>
+      <x:c r="B7" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C7" s="77" t="n">
+        <x:v>0.0995287356545802</x:v>
+      </x:c>
+      <x:c r="D7" s="77" t="n">
+        <x:v>0.17441678491295232</x:v>
+      </x:c>
+      <x:c r="E7" s="77" t="n">
+        <x:f>D7-C7</x:f>
+        <x:v>0.07488804925837211</x:v>
+      </x:c>
+      <x:c r="F7" s="77" t="n">
+        <x:v>0.2067137020942127</x:v>
+      </x:c>
+      <x:c r="G7" s="77" t="n">
+        <x:f>F7-C7</x:f>
+        <x:v>0.10718496643963249</x:v>
+      </x:c>
+      <x:c r="H7" s="77" t="n">
+        <x:v>0.16930032683497043</x:v>
+      </x:c>
+      <x:c r="I7" s="77" t="n">
+        <x:f>H7-C7</x:f>
+        <x:v>0.06977159118039022</x:v>
+      </x:c>
+      <x:c r="J7" s="77" t="n">
+        <x:v>0.17441678491295232</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="76" t="str">
+        <x:v>p04</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C8" s="77" t="n">
+        <x:v>1.2006884882495612</x:v>
+      </x:c>
+      <x:c r="D8" s="77" t="n">
+        <x:v>1.2068380536505807</x:v>
+      </x:c>
+      <x:c r="E8" s="77" t="n">
+        <x:f>D8-C8</x:f>
+        <x:v>0.006149565401019519</x:v>
+      </x:c>
+      <x:c r="F8" s="77" t="n">
+        <x:v>1.1830417047568231</x:v>
+      </x:c>
+      <x:c r="G8" s="77" t="n">
+        <x:f>F8-C8</x:f>
+        <x:v>-0.017646783492738072</x:v>
+      </x:c>
+      <x:c r="H8" s="77" t="n">
+        <x:v>1.2355777756943005</x:v>
+      </x:c>
+      <x:c r="I8" s="77" t="n">
+        <x:f>H8-C8</x:f>
+        <x:v>0.03488928744473929</x:v>
+      </x:c>
+      <x:c r="J8" s="77" t="n">
+        <x:v>1.2068380536505807</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="76" t="str">
+        <x:v>p05</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C9" s="77" t="n">
+        <x:v>1.6695828759409508</x:v>
+      </x:c>
+      <x:c r="D9" s="77" t="n">
+        <x:v>2.1473031919305465</x:v>
+      </x:c>
+      <x:c r="E9" s="77" t="n">
+        <x:f>D9-C9</x:f>
+        <x:v>0.47772031598959575</x:v>
+      </x:c>
+      <x:c r="F9" s="77" t="n">
+        <x:v>1.7442419771178912</x:v>
+      </x:c>
+      <x:c r="G9" s="77" t="n">
+        <x:f>F9-C9</x:f>
+        <x:v>0.07465910117694041</x:v>
+      </x:c>
+      <x:c r="H9" s="77" t="n">
+        <x:v>1.7093542588665314</x:v>
+      </x:c>
+      <x:c r="I9" s="77" t="n">
+        <x:f>H9-C9</x:f>
+        <x:v>0.03977138292558058</x:v>
+      </x:c>
+      <x:c r="J9" s="77" t="n">
+        <x:v>2.1473031919305465</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="76" t="str">
+        <x:v>p06</x:v>
+      </x:c>
+      <x:c r="B10" s="76" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C10" s="77" t="n">
+        <x:v>1.3459179912832273</x:v>
+      </x:c>
+      <x:c r="D10" s="77" t="n">
+        <x:v>1.1412870674482067</x:v>
+      </x:c>
+      <x:c r="E10" s="77" t="n">
+        <x:f>D10-C10</x:f>
+        <x:v>-0.20463092383502057</x:v>
+      </x:c>
+      <x:c r="F10" s="77" t="n">
+        <x:v>1.1175196348823742</x:v>
+      </x:c>
+      <x:c r="G10" s="77" t="n">
+        <x:f>F10-C10</x:f>
+        <x:v>-0.22839835640085315</x:v>
+      </x:c>
+      <x:c r="H10" s="77" t="n">
+        <x:v>1.1748173775503725</x:v>
+      </x:c>
+      <x:c r="I10" s="77" t="n">
+        <x:f>H10-C10</x:f>
+        <x:v>-0.1711006137328548</x:v>
+      </x:c>
+      <x:c r="J10" s="77" t="n">
+        <x:v>1.1412870674482067</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="76" t="str">
+        <x:v>p07</x:v>
+      </x:c>
+      <x:c r="B11" s="76" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="C11" s="77" t="n">
+        <x:v>1.7726823590623266</x:v>
+      </x:c>
+      <x:c r="D11" s="77" t="n">
+        <x:v>1.3551139161088712</x:v>
+      </x:c>
+      <x:c r="E11" s="77" t="n">
+        <x:f>D11-C11</x:f>
+        <x:v>-0.4175684429534554</x:v>
+      </x:c>
+      <x:c r="F11" s="77" t="n">
+        <x:v>1.3636408849210948</x:v>
+      </x:c>
+      <x:c r="G11" s="77" t="n">
+        <x:f>F11-C11</x:f>
+        <x:v>-0.4090414741412318</x:v>
+      </x:c>
+      <x:c r="H11" s="77" t="n">
+        <x:v>1.497051066688677</x:v>
+      </x:c>
+      <x:c r="I11" s="77" t="n">
+        <x:f>H11-C11</x:f>
+        <x:v>-0.2756312923736497</x:v>
+      </x:c>
+      <x:c r="J11" s="77" t="n">
+        <x:v>1.3551139161088712</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="76" t="str">
+        <x:v>p08</x:v>
+      </x:c>
+      <x:c r="B12" s="76" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C12" s="77" t="n">
+        <x:v>1.6467649477612443</x:v>
+      </x:c>
+      <x:c r="D12" s="77" t="n">
+        <x:v>1.331140876563422</x:v>
+      </x:c>
+      <x:c r="E12" s="77" t="n">
+        <x:f>D12-C12</x:f>
+        <x:v>-0.3156240711978222</x:v>
+      </x:c>
+      <x:c r="F12" s="77" t="n">
+        <x:v>1.361340228412525</x:v>
+      </x:c>
+      <x:c r="G12" s="77" t="n">
+        <x:f>F12-C12</x:f>
+        <x:v>-0.28542471934871916</x:v>
+      </x:c>
+      <x:c r="H12" s="77" t="n">
+        <x:v>1.465424185764665</x:v>
+      </x:c>
+      <x:c r="I12" s="77" t="n">
+        <x:f>H12-C12</x:f>
+        <x:v>-0.18134076199657923</x:v>
+      </x:c>
+      <x:c r="J12" s="77" t="n">
+        <x:v>1.331140876563422</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="76" t="str">
+        <x:v>p09</x:v>
+      </x:c>
+      <x:c r="B13" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C13" s="77" t="n">
+        <x:v>1.438914622426954</x:v>
+      </x:c>
+      <x:c r="D13" s="77" t="n">
+        <x:v>1.2271874632143245</x:v>
+      </x:c>
+      <x:c r="E13" s="77" t="n">
+        <x:f>D13-C13</x:f>
+        <x:v>-0.21172715921262952</x:v>
+      </x:c>
+      <x:c r="F13" s="77" t="n">
+        <x:v>1.2916569077966522</x:v>
+      </x:c>
+      <x:c r="G13" s="77" t="n">
+        <x:f>F13-C13</x:f>
+        <x:v>-0.1472577146303018</x:v>
+      </x:c>
+      <x:c r="H13" s="77" t="n">
+        <x:v>1.2454164814693112</x:v>
+      </x:c>
+      <x:c r="I13" s="77" t="n">
+        <x:f>H13-C13</x:f>
+        <x:v>-0.19349814095764284</x:v>
+      </x:c>
+      <x:c r="J13" s="77" t="n">
+        <x:v>1.4199796097549302</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="76" t="str">
+        <x:v>p10</x:v>
+      </x:c>
+      <x:c r="B14" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="77" t="n">
+        <x:v>3.2832124090462127</x:v>
+      </x:c>
+      <x:c r="D14" s="77" t="n">
+        <x:v>3.2762154161719366</x:v>
+      </x:c>
+      <x:c r="E14" s="77" t="n">
+        <x:f>D14-C14</x:f>
+        <x:v>-0.006996992874276131</x:v>
+      </x:c>
+      <x:c r="F14" s="77" t="n">
+        <x:v>3.356959243036494</x:v>
+      </x:c>
+      <x:c r="G14" s="77" t="n">
+        <x:f>F14-C14</x:f>
+        <x:v>0.07374683399028115</x:v>
+      </x:c>
+      <x:c r="H14" s="77" t="n">
+        <x:v>3.3493002558641862</x:v>
+      </x:c>
+      <x:c r="I14" s="77" t="n">
+        <x:f>H14-C14</x:f>
+        <x:v>0.06608784681797353</x:v>
+      </x:c>
+      <x:c r="J14" s="77" t="n">
+        <x:v>3.2762154161719366</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="76" t="str">
+        <x:v>p11</x:v>
+      </x:c>
+      <x:c r="B15" s="76" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C15" s="77" t="n">
+        <x:v>1.9373546513548079</x:v>
+      </x:c>
+      <x:c r="D15" s="77" t="n">
+        <x:v>1.72371580693681</x:v>
+      </x:c>
+      <x:c r="E15" s="77" t="n">
+        <x:f>D15-C15</x:f>
+        <x:v>-0.21363884441799796</x:v>
+      </x:c>
+      <x:c r="F15" s="77" t="n">
+        <x:v>1.7044267994994975</x:v>
+      </x:c>
+      <x:c r="G15" s="77" t="n">
+        <x:f>F15-C15</x:f>
+        <x:v>-0.2329278518553104</x:v>
+      </x:c>
+      <x:c r="H15" s="77" t="n">
+        <x:v>1.7749116904960978</x:v>
+      </x:c>
+      <x:c r="I15" s="77" t="n">
+        <x:f>H15-C15</x:f>
+        <x:v>-0.16244296085871013</x:v>
+      </x:c>
+      <x:c r="J15" s="77" t="n">
+        <x:v>1.72371580693681</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="76" t="str">
+        <x:v>p12</x:v>
+      </x:c>
+      <x:c r="B16" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C16" s="77" t="n">
+        <x:v>0.3805812828660011</x:v>
+      </x:c>
+      <x:c r="D16" s="77" t="n">
+        <x:v>0.2714568794802408</x:v>
+      </x:c>
+      <x:c r="E16" s="77" t="n">
+        <x:f>D16-C16</x:f>
+        <x:v>-0.10912440338576035</x:v>
+      </x:c>
+      <x:c r="F16" s="77" t="n">
+        <x:v>0.2820074357868543</x:v>
+      </x:c>
+      <x:c r="G16" s="77" t="n">
+        <x:f>F16-C16</x:f>
+        <x:v>-0.09857384707914685</x:v>
+      </x:c>
+      <x:c r="H16" s="77" t="n">
+        <x:v>0.1730025095471892</x:v>
+      </x:c>
+      <x:c r="I16" s="77" t="n">
+        <x:f>H16-C16</x:f>
+        <x:v>-0.20757877331881192</x:v>
+      </x:c>
+      <x:c r="J16" s="77" t="n">
+        <x:v>0.2714568794802408</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="76" t="str">
+        <x:v>p13</x:v>
+      </x:c>
+      <x:c r="B17" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C17" s="77" t="n">
+        <x:v>0.7990183786925269</x:v>
+      </x:c>
+      <x:c r="D17" s="77" t="n">
+        <x:v>0.9587573389944235</x:v>
+      </x:c>
+      <x:c r="E17" s="77" t="n">
+        <x:f>D17-C17</x:f>
+        <x:v>0.1597389603018966</x:v>
+      </x:c>
+      <x:c r="F17" s="77" t="n">
+        <x:v>0.9667511075508379</x:v>
+      </x:c>
+      <x:c r="G17" s="77" t="n">
+        <x:f>F17-C17</x:f>
+        <x:v>0.16773272885831103</x:v>
+      </x:c>
+      <x:c r="H17" s="77" t="n">
+        <x:v>0.8592712610970663</x:v>
+      </x:c>
+      <x:c r="I17" s="77" t="n">
+        <x:f>H17-C17</x:f>
+        <x:v>0.06025288240453941</x:v>
+      </x:c>
+      <x:c r="J17" s="77" t="n">
+        <x:v>0.9587573389944235</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="76" t="str">
+        <x:v>p14</x:v>
+      </x:c>
+      <x:c r="B18" s="76" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C18" s="77" t="n">
+        <x:v>0.7577866369295649</x:v>
+      </x:c>
+      <x:c r="D18" s="77" t="n">
+        <x:v>0.653035042472271</x:v>
+      </x:c>
+      <x:c r="E18" s="77" t="n">
+        <x:f>D18-C18</x:f>
+        <x:v>-0.10475159445729398</x:v>
+      </x:c>
+      <x:c r="F18" s="77" t="n">
+        <x:v>0.6909513561227043</x:v>
+      </x:c>
+      <x:c r="G18" s="77" t="n">
+        <x:f>F18-C18</x:f>
+        <x:v>-0.06683528080686063</x:v>
+      </x:c>
+      <x:c r="H18" s="77" t="n">
+        <x:v>0.6517975489339697</x:v>
+      </x:c>
+      <x:c r="I18" s="77" t="n">
+        <x:f>H18-C18</x:f>
+        <x:v>-0.10598908799559525</x:v>
+      </x:c>
+      <x:c r="J18" s="77" t="n">
+        <x:v>0.653035042472271</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="76" t="str">
+        <x:v>p15</x:v>
+      </x:c>
+      <x:c r="B19" s="76" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C19" s="77" t="n">
+        <x:v>1.9214974186959535</x:v>
+      </x:c>
+      <x:c r="D19" s="77" t="n">
+        <x:v>1.8126158883083692</x:v>
+      </x:c>
+      <x:c r="E19" s="77" t="n">
+        <x:f>D19-C19</x:f>
+        <x:v>-0.1088815303875843</x:v>
+      </x:c>
+      <x:c r="F19" s="77" t="n">
+        <x:v>1.9044758992743513</x:v>
+      </x:c>
+      <x:c r="G19" s="77" t="n">
+        <x:f>F19-C19</x:f>
+        <x:v>-0.017021519421602127</x:v>
+      </x:c>
+      <x:c r="H19" s="77" t="n">
+        <x:v>1.8744105611659267</x:v>
+      </x:c>
+      <x:c r="I19" s="77" t="n">
+        <x:f>H19-C19</x:f>
+        <x:v>-0.04708685753002673</x:v>
+      </x:c>
+      <x:c r="J19" s="77" t="n">
+        <x:v>1.8126158883083692</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="B21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="C21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="D21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="E21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="F21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="G21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="H21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="I21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+      <x:c r="J21" s="81" t="str">
+        <x:v>Source file: analysis/reviewer_round5_participant_losses.csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A21:J21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="B1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="C1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="D1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="E1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+      <x:c r="F1" s="67" t="str">
+        <x:v>PMData sample-flow reconciliation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+      <x:c r="F2" s="70" t="str">
+        <x:v>Sequential construction and rule-specific reconstructions are separated because rematching can admit newly eligible pairs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>stage</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>sessions</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>definition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="76" t="str">
+        <x:v>Archived PMSys RPE records</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="n">
+        <x:v>783</x:v>
+      </x:c>
+      <x:c r="C5" s="76" t="str">
+        <x:v>all archived RPE rows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="76" t="str">
+        <x:v>Broad tracker-linked pairs</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="n">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="C6" s="76" t="str">
+        <x:v>timestamp and activity-compatible links</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="76" t="str">
+        <x:v>Bidirectionally unique broad pairs</x:v>
+      </x:c>
+      <x:c r="B7" s="76" t="n">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="C7" s="76" t="str">
+        <x:v>unique in both matching directions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="76" t="str">
+        <x:v>Unique broad pairs passing HR quality control</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="n">
+        <x:v>267</x:v>
+      </x:c>
+      <x:c r="C8" s="76" t="str">
+        <x:v>heart-rate signal criteria satisfied</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="76" t="str">
+        <x:v>Primary analysis sessions</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="C9" s="76" t="str">
+        <x:v>all primary matching and outcome criteria satisfied</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="82" t="str">
+        <x:v>Rule-specific matching sensitivity</x:v>
+      </x:c>
+      <x:c r="B12" s="82"/>
+      <x:c r="C12" s="82"/>
+      <x:c r="D12" s="82"/>
+      <x:c r="E12" s="82"/>
+      <x:c r="F12" s="82"/>
+    </x:row>
+    <x:row r="13" ht="32" customHeight="1">
+      <x:c r="A13" s="75" t="str">
+        <x:v>rule</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>selected_pairs</x:v>
+      </x:c>
+      <x:c r="C13" s="75" t="str">
+        <x:v>bidirectionally_unique_pairs</x:v>
+      </x:c>
+      <x:c r="D13" s="75" t="str">
+        <x:v>original_primary_pairs_retained</x:v>
+      </x:c>
+      <x:c r="E13" s="75" t="str">
+        <x:v>rebuilt_analysis_sessions</x:v>
+      </x:c>
+      <x:c r="F13" s="75" t="str">
+        <x:v>interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="76" t="str">
+        <x:v>Primary 15-180 min</x:v>
+      </x:c>
+      <x:c r="B14" s="76" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="C14" s="76" t="n">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="D14" s="76" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="E14" s="76" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="F14" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="76" t="str">
+        <x:v>15-90 min</x:v>
+      </x:c>
+      <x:c r="B15" s="76" t="n">
+        <x:v>401</x:v>
+      </x:c>
+      <x:c r="C15" s="76" t="n">
+        <x:v>398</x:v>
+      </x:c>
+      <x:c r="D15" s="76" t="n">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="E15" s="76" t="n">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="F15" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="76" t="str">
+        <x:v>30-120 min</x:v>
+      </x:c>
+      <x:c r="B16" s="76" t="n">
+        <x:v>413</x:v>
+      </x:c>
+      <x:c r="C16" s="76" t="n">
+        <x:v>408</x:v>
+      </x:c>
+      <x:c r="D16" s="76" t="n">
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="E16" s="76" t="n">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="F16" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="76" t="str">
+        <x:v>Duration difference &lt;=10 min</x:v>
+      </x:c>
+      <x:c r="B17" s="76" t="n">
+        <x:v>363</x:v>
+      </x:c>
+      <x:c r="C17" s="76" t="n">
+        <x:v>357</x:v>
+      </x:c>
+      <x:c r="D17" s="76" t="n">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="E17" s="76" t="n">
+        <x:v>220</x:v>
+      </x:c>
+      <x:c r="F17" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="76" t="str">
+        <x:v>Delay-priority cost</x:v>
+      </x:c>
+      <x:c r="B18" s="76" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="C18" s="76" t="n">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="D18" s="76" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="E18" s="76" t="n">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="F18" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="76" t="str">
+        <x:v>Duration-priority cost</x:v>
+      </x:c>
+      <x:c r="B19" s="76" t="n">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="C19" s="76" t="n">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="D19" s="76" t="n">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="E19" s="76" t="n">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="F19" s="76" t="str">
+        <x:v>Retained counts track IDs from the 255-session primary set; rebuilt counts include newly eligible matches after the rule-specific reconstruction and full quality control.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" customHeight="1">
+      <x:c r="A21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+      <x:c r="B21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+      <x:c r="C21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+      <x:c r="D21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+      <x:c r="E21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+      <x:c r="F21" s="81" t="str">
+        <x:v>Source files: analysis/reviewer_round5_primary_sample_flow.csv and analysis/reviewer_round5_sensitivity_sample_flow.csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A2:F2"/>
+    <x:mergeCell ref="A12:F12"/>
+    <x:mergeCell ref="A21:F21"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="17" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="17" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="17" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="17" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="17" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="B1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="C1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="D1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="E1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="F1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="G1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="H1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="I1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="J1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="K1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="L1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="M1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="N1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="O1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="P1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="Q1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="R1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="S1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="T1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+      <x:c r="U1" s="67" t="str">
+        <x:v>WEEE repeated-measures agreement</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="F2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="G2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="H2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="I2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="J2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="K2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="L2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="M2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="N2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="O2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="P2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="Q2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="R2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="S2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="T2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+      <x:c r="U2" s="70" t="str">
+        <x:v>Primary manuscript inference uses Zephyr (16 participants, 77 stages). Apple Watch and E4 rows are retained only to disclose inadequate participant coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>Device</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>Participants</x:v>
+      </x:c>
+      <x:c r="D4" s="75" t="str">
+        <x:v>Stages</x:v>
+      </x:c>
+      <x:c r="E4" s="75" t="str">
+        <x:v>Balanced bias</x:v>
+      </x:c>
+      <x:c r="F4" s="75" t="str">
+        <x:v>Between-person difference variance</x:v>
+      </x:c>
+      <x:c r="G4" s="75" t="str">
+        <x:v>Within-person difference variance</x:v>
+      </x:c>
+      <x:c r="H4" s="75" t="str">
+        <x:v>RM LoA lower</x:v>
+      </x:c>
+      <x:c r="I4" s="75" t="str">
+        <x:v>RM LoA upper</x:v>
+      </x:c>
+      <x:c r="J4" s="75" t="str">
+        <x:v>Balanced CCC</x:v>
+      </x:c>
+      <x:c r="K4" s="75" t="str">
+        <x:v>Participant-centered r</x:v>
+      </x:c>
+      <x:c r="L4" s="75" t="str">
+        <x:v>Bias CI lower</x:v>
+      </x:c>
+      <x:c r="M4" s="75" t="str">
+        <x:v>Bias CI upper</x:v>
+      </x:c>
+      <x:c r="N4" s="75" t="str">
+        <x:v>LoA lower CI lower</x:v>
+      </x:c>
+      <x:c r="O4" s="75" t="str">
+        <x:v>LoA lower CI upper</x:v>
+      </x:c>
+      <x:c r="P4" s="75" t="str">
+        <x:v>LoA upper CI lower</x:v>
+      </x:c>
+      <x:c r="Q4" s="75" t="str">
+        <x:v>LoA upper CI upper</x:v>
+      </x:c>
+      <x:c r="R4" s="75" t="str">
+        <x:v>CCC CI lower</x:v>
+      </x:c>
+      <x:c r="S4" s="75" t="str">
+        <x:v>CCC CI upper</x:v>
+      </x:c>
+      <x:c r="T4" s="75" t="str">
+        <x:v>Centered r CI lower</x:v>
+      </x:c>
+      <x:c r="U4" s="75" t="str">
+        <x:v>Centered r CI upper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="76" t="str">
+        <x:v>apple_watch</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="str">
+        <x:v>mean_hrr</x:v>
+      </x:c>
+      <x:c r="C5" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D5" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E5" s="77" t="n">
+        <x:v>-0.42749684422358447</x:v>
+      </x:c>
+      <x:c r="F5" s="77"/>
+      <x:c r="G5" s="77" t="n">
+        <x:v>0.00701739666078539</x:v>
+      </x:c>
+      <x:c r="H5" s="77"/>
+      <x:c r="I5" s="77"/>
+      <x:c r="J5" s="77" t="n">
+        <x:v>0.004394910473526646</x:v>
+      </x:c>
+      <x:c r="K5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L5" s="77" t="n">
+        <x:v>-0.42749684422358447</x:v>
+      </x:c>
+      <x:c r="M5" s="77" t="n">
+        <x:v>-0.42749684422358447</x:v>
+      </x:c>
+      <x:c r="N5" s="77"/>
+      <x:c r="O5" s="77"/>
+      <x:c r="P5" s="77"/>
+      <x:c r="Q5" s="77"/>
+      <x:c r="R5" s="77" t="n">
+        <x:v>0.004394910473526646</x:v>
+      </x:c>
+      <x:c r="S5" s="77" t="n">
+        <x:v>0.004394910473526646</x:v>
+      </x:c>
+      <x:c r="T5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U5" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="76" t="str">
+        <x:v>apple_watch</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="str">
+        <x:v>thrr_i</x:v>
+      </x:c>
+      <x:c r="C6" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E6" s="77" t="n">
+        <x:v>-0.4120317476714055</x:v>
+      </x:c>
+      <x:c r="F6" s="77"/>
+      <x:c r="G6" s="77" t="n">
+        <x:v>0.009276650435766006</x:v>
+      </x:c>
+      <x:c r="H6" s="77"/>
+      <x:c r="I6" s="77"/>
+      <x:c r="J6" s="77" t="n">
+        <x:v>0.006287974137288232</x:v>
+      </x:c>
+      <x:c r="K6" s="77" t="n">
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+      <x:c r="L6" s="77" t="n">
+        <x:v>-0.4120317476714055</x:v>
+      </x:c>
+      <x:c r="M6" s="77" t="n">
+        <x:v>-0.4120317476714055</x:v>
+      </x:c>
+      <x:c r="N6" s="77"/>
+      <x:c r="O6" s="77"/>
+      <x:c r="P6" s="77"/>
+      <x:c r="Q6" s="77"/>
+      <x:c r="R6" s="77" t="n">
+        <x:v>0.006287974137288232</x:v>
+      </x:c>
+      <x:c r="S6" s="77" t="n">
+        <x:v>0.006287974137288232</x:v>
+      </x:c>
+      <x:c r="T6" s="77" t="n">
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+      <x:c r="U6" s="77" t="n">
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="76" t="str">
+        <x:v>apple_watch</x:v>
+      </x:c>
+      <x:c r="B7" s="76" t="str">
+        <x:v>delta_tilt</x:v>
+      </x:c>
+      <x:c r="C7" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D7" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E7" s="77" t="n">
+        <x:v>0.01546509655217905</x:v>
+      </x:c>
+      <x:c r="F7" s="77"/>
+      <x:c r="G7" s="77" t="n">
+        <x:v>0.00015738873229050808</x:v>
+      </x:c>
+      <x:c r="H7" s="77"/>
+      <x:c r="I7" s="77"/>
+      <x:c r="J7" s="77" t="n">
+        <x:v>0.06095116141173844</x:v>
+      </x:c>
+      <x:c r="K7" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L7" s="77" t="n">
+        <x:v>0.01546509655217905</x:v>
+      </x:c>
+      <x:c r="M7" s="77" t="n">
+        <x:v>0.01546509655217905</x:v>
+      </x:c>
+      <x:c r="N7" s="77"/>
+      <x:c r="O7" s="77"/>
+      <x:c r="P7" s="77"/>
+      <x:c r="Q7" s="77"/>
+      <x:c r="R7" s="77" t="n">
+        <x:v>0.06095116141173844</x:v>
+      </x:c>
+      <x:c r="S7" s="77" t="n">
+        <x:v>0.06095116141173844</x:v>
+      </x:c>
+      <x:c r="T7" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="U7" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="76" t="str">
+        <x:v>e4</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="str">
+        <x:v>mean_hrr</x:v>
+      </x:c>
+      <x:c r="C8" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D8" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E8" s="77" t="n">
+        <x:v>0.011972552195592234</x:v>
+      </x:c>
+      <x:c r="F8" s="77" t="n">
+        <x:v>0.07758612098469439</x:v>
+      </x:c>
+      <x:c r="G8" s="77" t="n">
+        <x:v>0.009621295097330819</x:v>
+      </x:c>
+      <x:c r="H8" s="77" t="n">
+        <x:v>-0.566833122984522</x:v>
+      </x:c>
+      <x:c r="I8" s="77" t="n">
+        <x:v>0.5907782273757065</x:v>
+      </x:c>
+      <x:c r="J8" s="77" t="n">
+        <x:v>-0.28400163814416163</x:v>
+      </x:c>
+      <x:c r="K8" s="77" t="n">
+        <x:v>0.7242072426030246</x:v>
+      </x:c>
+      <x:c r="L8" s="77" t="n">
+        <x:v>-0.19100129899386492</x:v>
+      </x:c>
+      <x:c r="M8" s="77" t="n">
+        <x:v>0.2149464033850494</x:v>
+      </x:c>
+      <x:c r="N8" s="77" t="n">
+        <x:v>-0.566833122984522</x:v>
+      </x:c>
+      <x:c r="O8" s="77" t="n">
+        <x:v>-0.006063381541955376</x:v>
+      </x:c>
+      <x:c r="P8" s="77" t="n">
+        <x:v>-0.03264407794496155</x:v>
+      </x:c>
+      <x:c r="Q8" s="77" t="n">
+        <x:v>0.5907782273757065</x:v>
+      </x:c>
+      <x:c r="R8" s="77" t="n">
+        <x:v>-0.28400163814416163</x:v>
+      </x:c>
+      <x:c r="S8" s="77" t="n">
+        <x:v>0.026880214821956898</x:v>
+      </x:c>
+      <x:c r="T8" s="77" t="n">
+        <x:v>0.7242072426030246</x:v>
+      </x:c>
+      <x:c r="U8" s="77" t="n">
+        <x:v>1.0000000000000002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="76" t="str">
+        <x:v>e4</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="str">
+        <x:v>thrr_i</x:v>
+      </x:c>
+      <x:c r="C9" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D9" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E9" s="77" t="n">
+        <x:v>0.29759352624063135</x:v>
+      </x:c>
+      <x:c r="F9" s="77" t="n">
+        <x:v>0.2966176427432425</x:v>
+      </x:c>
+      <x:c r="G9" s="77" t="n">
+        <x:v>0.016262330770474</x:v>
+      </x:c>
+      <x:c r="H9" s="77" t="n">
+        <x:v>-0.7987457033093712</x:v>
+      </x:c>
+      <x:c r="I9" s="77" t="n">
+        <x:v>1.3939327557906338</x:v>
+      </x:c>
+      <x:c r="J9" s="77" t="n">
+        <x:v>-0.44398257057384943</x:v>
+      </x:c>
+      <x:c r="K9" s="77" t="n">
+        <x:v>-0.855734879751444</x:v>
+      </x:c>
+      <x:c r="L9" s="77" t="n">
+        <x:v>-0.09275811531380065</x:v>
+      </x:c>
+      <x:c r="M9" s="77" t="n">
+        <x:v>0.6879451677950633</x:v>
+      </x:c>
+      <x:c r="N9" s="77" t="n">
+        <x:v>-0.7987457033093712</x:v>
+      </x:c>
+      <x:c r="O9" s="77" t="n">
+        <x:v>0.47742423168987336</x:v>
+      </x:c>
+      <x:c r="P9" s="77" t="n">
+        <x:v>0.19119201276699513</x:v>
+      </x:c>
+      <x:c r="Q9" s="77" t="n">
+        <x:v>1.3939327557906338</x:v>
+      </x:c>
+      <x:c r="R9" s="77" t="n">
+        <x:v>-0.4439825705738496</x:v>
+      </x:c>
+      <x:c r="S9" s="77" t="n">
+        <x:v>-0.0016629031813126896</x:v>
+      </x:c>
+      <x:c r="T9" s="77" t="n">
+        <x:v>-1.0000000000000002</x:v>
+      </x:c>
+      <x:c r="U9" s="77" t="n">
+        <x:v>-0.855734879751444</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="76" t="str">
+        <x:v>e4</x:v>
+      </x:c>
+      <x:c r="B10" s="76" t="str">
+        <x:v>delta_tilt</x:v>
+      </x:c>
+      <x:c r="C10" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D10" s="76" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E10" s="77" t="n">
+        <x:v>0.28562097404503906</x:v>
+      </x:c>
+      <x:c r="F10" s="77" t="n">
+        <x:v>0.0691872151676574</x:v>
+      </x:c>
+      <x:c r="G10" s="77" t="n">
+        <x:v>0.0020673149529269606</x:v>
+      </x:c>
+      <x:c r="H10" s="77" t="n">
+        <x:v>-0.23757249199905905</x:v>
+      </x:c>
+      <x:c r="I10" s="77" t="n">
+        <x:v>0.8088144400891372</x:v>
+      </x:c>
+      <x:c r="J10" s="77" t="n">
+        <x:v>0.023929760286168326</x:v>
+      </x:c>
+      <x:c r="K10" s="77" t="n">
+        <x:v>-0.5372571806320987</x:v>
+      </x:c>
+      <x:c r="L10" s="77" t="n">
+        <x:v>0.0982431836800643</x:v>
+      </x:c>
+      <x:c r="M10" s="77" t="n">
+        <x:v>0.47299876441001387</x:v>
+      </x:c>
+      <x:c r="N10" s="77" t="n">
+        <x:v>-0.23757249199905905</x:v>
+      </x:c>
+      <x:c r="O10" s="77" t="n">
+        <x:v>0.462509915588199</x:v>
+      </x:c>
+      <x:c r="P10" s="77" t="n">
+        <x:v>0.22383609071195656</x:v>
+      </x:c>
+      <x:c r="Q10" s="77" t="n">
+        <x:v>0.8088144400891372</x:v>
+      </x:c>
+      <x:c r="R10" s="77" t="n">
+        <x:v>-0.06377508034879854</x:v>
+      </x:c>
+      <x:c r="S10" s="77" t="n">
+        <x:v>0.023929760286168326</x:v>
+      </x:c>
+      <x:c r="T10" s="77" t="n">
+        <x:v>-1</x:v>
+      </x:c>
+      <x:c r="U10" s="77" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="76" t="str">
+        <x:v>zephyr</x:v>
+      </x:c>
+      <x:c r="B11" s="76" t="str">
+        <x:v>mean_hrr</x:v>
+      </x:c>
+      <x:c r="C11" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D11" s="76" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E11" s="77" t="n">
+        <x:v>-0.024858046793567373</x:v>
+      </x:c>
+      <x:c r="F11" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G11" s="77" t="n">
+        <x:v>0.006391080674646548</x:v>
+      </x:c>
+      <x:c r="H11" s="77" t="n">
+        <x:v>-0.18154874696343126</x:v>
+      </x:c>
+      <x:c r="I11" s="77" t="n">
+        <x:v>0.13183265337629652</x:v>
+      </x:c>
+      <x:c r="J11" s="77" t="n">
+        <x:v>0.9168775264083271</x:v>
+      </x:c>
+      <x:c r="K11" s="77" t="n">
+        <x:v>0.9251380220583476</x:v>
+      </x:c>
+      <x:c r="L11" s="77" t="n">
+        <x:v>-0.036574906398400824</x:v>
+      </x:c>
+      <x:c r="M11" s="77" t="n">
+        <x:v>-0.009774815512390915</x:v>
+      </x:c>
+      <x:c r="N11" s="77" t="n">
+        <x:v>-0.24566620822728918</x:v>
+      </x:c>
+      <x:c r="O11" s="77" t="n">
+        <x:v>-0.10342762140728763</x:v>
+      </x:c>
+      <x:c r="P11" s="77" t="n">
+        <x:v>0.046756936136455214</x:v>
+      </x:c>
+      <x:c r="Q11" s="77" t="n">
+        <x:v>0.2170832678898023</x:v>
+      </x:c>
+      <x:c r="R11" s="77" t="n">
+        <x:v>0.7856849470521989</x:v>
+      </x:c>
+      <x:c r="S11" s="77" t="n">
+        <x:v>0.9740243291474556</x:v>
+      </x:c>
+      <x:c r="T11" s="77" t="n">
+        <x:v>0.7766037370296658</x:v>
+      </x:c>
+      <x:c r="U11" s="77" t="n">
+        <x:v>0.9908622143407204</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="76" t="str">
+        <x:v>zephyr</x:v>
+      </x:c>
+      <x:c r="B12" s="76" t="str">
+        <x:v>thrr_i</x:v>
+      </x:c>
+      <x:c r="C12" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D12" s="76" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E12" s="77" t="n">
+        <x:v>-0.024566717840435154</x:v>
+      </x:c>
+      <x:c r="F12" s="77" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="77" t="n">
+        <x:v>0.014720217621991667</x:v>
+      </x:c>
+      <x:c r="H12" s="77" t="n">
+        <x:v>-0.2623674495816205</x:v>
+      </x:c>
+      <x:c r="I12" s="77" t="n">
+        <x:v>0.21323401390075017</x:v>
+      </x:c>
+      <x:c r="J12" s="77" t="n">
+        <x:v>0.8464359139148857</x:v>
+      </x:c>
+      <x:c r="K12" s="77" t="n">
+        <x:v>0.8464336809580291</x:v>
+      </x:c>
+      <x:c r="L12" s="77" t="n">
+        <x:v>-0.04391137019111345</x:v>
+      </x:c>
+      <x:c r="M12" s="77" t="n">
+        <x:v>-0.000738936223250524</x:v>
+      </x:c>
+      <x:c r="N12" s="77" t="n">
+        <x:v>-0.33901136050163794</x:v>
+      </x:c>
+      <x:c r="O12" s="77" t="n">
+        <x:v>-0.16119469532749045</x:v>
+      </x:c>
+      <x:c r="P12" s="77" t="n">
+        <x:v>0.08406097320493748</x:v>
+      </x:c>
+      <x:c r="Q12" s="77" t="n">
+        <x:v>0.32906587348297317</x:v>
+      </x:c>
+      <x:c r="R12" s="77" t="n">
+        <x:v>0.6541604454054335</x:v>
+      </x:c>
+      <x:c r="S12" s="77" t="n">
+        <x:v>0.9464125755630209</x:v>
+      </x:c>
+      <x:c r="T12" s="77" t="n">
+        <x:v>0.6495393524359105</x:v>
+      </x:c>
+      <x:c r="U12" s="77" t="n">
+        <x:v>0.9709472840972481</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="76" t="str">
+        <x:v>zephyr</x:v>
+      </x:c>
+      <x:c r="B13" s="76" t="str">
+        <x:v>delta_tilt</x:v>
+      </x:c>
+      <x:c r="C13" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D13" s="76" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E13" s="77" t="n">
+        <x:v>0.0002913289531322333</x:v>
+      </x:c>
+      <x:c r="F13" s="77" t="n">
+        <x:v>0.0001166982479605607</x:v>
+      </x:c>
+      <x:c r="G13" s="77" t="n">
+        <x:v>0.003207664959121301</x:v>
+      </x:c>
+      <x:c r="H13" s="77" t="n">
+        <x:v>-0.11271696143445693</x:v>
+      </x:c>
+      <x:c r="I13" s="77" t="n">
+        <x:v>0.1132996193407214</x:v>
+      </x:c>
+      <x:c r="J13" s="77" t="n">
+        <x:v>0.15640098297953384</x:v>
+      </x:c>
+      <x:c r="K13" s="77" t="n">
+        <x:v>0.17069049468212721</x:v>
+      </x:c>
+      <x:c r="L13" s="77" t="n">
+        <x:v>-0.01206018189894072</x:v>
+      </x:c>
+      <x:c r="M13" s="77" t="n">
+        <x:v>0.013920896408066477</x:v>
+      </x:c>
+      <x:c r="N13" s="77" t="n">
+        <x:v>-0.15184641188540243</x:v>
+      </x:c>
+      <x:c r="O13" s="77" t="n">
+        <x:v>-0.07248837209209001</x:v>
+      </x:c>
+      <x:c r="P13" s="77" t="n">
+        <x:v>0.0547118433665161</x:v>
+      </x:c>
+      <x:c r="Q13" s="77" t="n">
+        <x:v>0.1656540355948107</x:v>
+      </x:c>
+      <x:c r="R13" s="77" t="n">
+        <x:v>-0.006627259837690882</x:v>
+      </x:c>
+      <x:c r="S13" s="77" t="n">
+        <x:v>0.4669120906883816</x:v>
+      </x:c>
+      <x:c r="T13" s="77" t="n">
+        <x:v>-0.05321895299303002</x:v>
+      </x:c>
+      <x:c r="U13" s="77" t="n">
+        <x:v>0.5545165220140845</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" customHeight="1">
+      <x:c r="A15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="B15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="C15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="D15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="E15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="F15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="G15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="H15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="I15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="J15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="K15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="L15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="M15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="N15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="O15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="P15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="Q15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="R15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="S15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="T15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+      <x:c r="U15" s="81" t="str">
+        <x:v>Source file: external_validation/results/reviewer_round5_weee_repeated_agreement.csv | Public data: https://doi.org/10.5281/zenodo.6420886</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:U1"/>
+    <x:mergeCell ref="A2:U2"/>
+    <x:mergeCell ref="A15:U15"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="62" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="67" t="str">
+        <x:v>WEEE participant and stage attrition</x:v>
+      </x:c>
+      <x:c r="B1" s="67" t="str">
+        <x:v>WEEE participant and stage attrition</x:v>
+      </x:c>
+      <x:c r="C1" s="67" t="str">
+        <x:v>WEEE participant and stage attrition</x:v>
+      </x:c>
+      <x:c r="D1" s="67" t="str">
+        <x:v>WEEE participant and stage attrition</x:v>
+      </x:c>
+      <x:c r="E1" s="67" t="str">
+        <x:v>WEEE participant and stage attrition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="70" t="str">
+        <x:v>High-running-stage retention was 3/16 (18.8%); this intensity-dependent attrition limits upper-tail inference.</x:v>
+      </x:c>
+      <x:c r="B2" s="70" t="str">
+        <x:v>High-running-stage retention was 3/16 (18.8%); this intensity-dependent attrition limits upper-tail inference.</x:v>
+      </x:c>
+      <x:c r="C2" s="70" t="str">
+        <x:v>High-running-stage retention was 3/16 (18.8%); this intensity-dependent attrition limits upper-tail inference.</x:v>
+      </x:c>
+      <x:c r="D2" s="70" t="str">
+        <x:v>High-running-stage retention was 3/16 (18.8%); this intensity-dependent attrition limits upper-tail inference.</x:v>
+      </x:c>
+      <x:c r="E2" s="70" t="str">
+        <x:v>High-running-stage retention was 3/16 (18.8%); this intensity-dependent attrition limits upper-tail inference.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="32" customHeight="1">
+      <x:c r="A4" s="75" t="str">
+        <x:v>stage</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>eligible_after_anchor_qc</x:v>
+      </x:c>
+      <x:c r="C4" s="75" t="str">
+        <x:v>included</x:v>
+      </x:c>
+      <x:c r="D4" s="75" t="str">
+        <x:v>excluded_stage_qc</x:v>
+      </x:c>
+      <x:c r="E4" s="75" t="str">
+        <x:v>retention_percent</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="76" t="str">
+        <x:v>sit</x:v>
+      </x:c>
+      <x:c r="B5" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C5" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D5" s="76" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E5" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="76" t="str">
+        <x:v>stand</x:v>
+      </x:c>
+      <x:c r="B6" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C6" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D6" s="76" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E6" s="78" t="n">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="76" t="str">
+        <x:v>cycle_low</x:v>
+      </x:c>
+      <x:c r="B7" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C7" s="76" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D7" s="76" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E7" s="78" t="n">
+        <x:v>93.75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="76" t="str">
+        <x:v>cycle_high</x:v>
+      </x:c>
+      <x:c r="B8" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C8" s="76" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D8" s="76" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E8" s="78" t="n">
+        <x:v>87.5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="76" t="str">
+        <x:v>run_low</x:v>
+      </x:c>
+      <x:c r="B9" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C9" s="76" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D9" s="76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E9" s="78" t="n">
+        <x:v>81.25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="76" t="str">
+        <x:v>run_high</x:v>
+      </x:c>
+      <x:c r="B10" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C10" s="76" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="76" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E10" s="78" t="n">
+        <x:v>18.75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="32" customHeight="1">
+      <x:c r="A13" s="75" t="str">
+        <x:v>flow_stage</x:v>
+      </x:c>
+      <x:c r="B13" s="75" t="str">
+        <x:v>participants</x:v>
+      </x:c>
+      <x:c r="C13" s="75" t="str">
+        <x:v>participant_stages</x:v>
+      </x:c>
+      <x:c r="D13" s="75" t="str">
+        <x:v>reason</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="76" t="str">
+        <x:v>Source participants</x:v>
+      </x:c>
+      <x:c r="B14" s="76" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C14" s="76" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="D14" s="76" t="str">
+        <x:v>17 participants x 6 protocol stages</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="76" t="str">
+        <x:v>Participants with resting-HR anchor</x:v>
+      </x:c>
+      <x:c r="B15" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C15" s="76" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="D15" s="76" t="str">
+        <x:v>P10 excluded because the sitting anchor was missing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="76" t="str">
+        <x:v>Final construct-analysis sample</x:v>
+      </x:c>
+      <x:c r="B16" s="76" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C16" s="76" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D16" s="76" t="str">
+        <x:v>19 additional participant-stage records failed reference HR or VO2 coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" customHeight="1">
+      <x:c r="A18" s="81" t="str">
+        <x:v>Source files: external_validation/results/reviewer_round5_weee_stage_flow.csv and reviewer_round5_weee_participant_flow.csv</x:v>
+      </x:c>
+      <x:c r="B18" s="81" t="str">
+        <x:v>Source files: external_validation/results/reviewer_round5_weee_stage_flow.csv and reviewer_round5_weee_participant_flow.csv</x:v>
+      </x:c>
+      <x:c r="C18" s="81" t="str">
+        <x:v>Source files: external_validation/results/reviewer_round5_weee_stage_flow.csv and reviewer_round5_weee_participant_flow.csv</x:v>
+      </x:c>
+      <x:c r="D18" s="81" t="str">
+        <x:v>Source files: external_validation/results/reviewer_round5_weee_stage_flow.csv and reviewer_round5_weee_participant_flow.csv</x:v>
+      </x:c>
+      <x:c r="E18" s="81" t="str">
+        <x:v>Source files: external_validation/results/reviewer_round5_weee_stage_flow.csv and reviewer_round5_weee_participant_flow.csv</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A18:E18"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>